<commit_message>
Update THÁNG 3.2026- CHÂU NGÂN- ĐỐI SOÁT.xlsx
</commit_message>
<xml_diff>
--- a/data/Mar/THÁNG 3.2026- CHÂU NGÂN- ĐỐI SOÁT.xlsx
+++ b/data/Mar/THÁNG 3.2026- CHÂU NGÂN- ĐỐI SOÁT.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Freelance\TextInputter\data\Mar\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\TextExtractorTool\data\Mar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A39F124-B57A-4BAF-A501-5F19BF2E5EBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C394BEC9-5214-47A1-8F36-F2F45D37C947}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="16" xr2:uid="{5C19E60F-B0EA-4466-8994-298A0AC29210}"/>
+    <workbookView xWindow="-28920" yWindow="-150" windowWidth="29040" windowHeight="15720" activeTab="10" xr2:uid="{5C19E60F-B0EA-4466-8994-298A0AC29210}"/>
   </bookViews>
   <sheets>
     <sheet name="2-3" sheetId="1" r:id="rId1"/>
@@ -6571,7 +6571,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -6623,8 +6623,7 @@
     <xf numFmtId="3" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="1" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="1" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -25295,7 +25294,9 @@
       <c r="Q5" s="25">
         <v>1</v>
       </c>
-      <c r="R5" s="25"/>
+      <c r="R5" s="25">
+        <v>30</v>
+      </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="21"/>
@@ -26221,59 +26222,59 @@
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.25">
       <c r="G28">
-        <f>SUBTOTAL(9,G3:G27)</f>
+        <f t="shared" ref="G28:R28" si="0">SUBTOTAL(9,G3:G27)</f>
         <v>9385</v>
       </c>
       <c r="H28">
-        <f>SUBTOTAL(9,H3:H27)</f>
+        <f t="shared" si="0"/>
         <v>655</v>
       </c>
       <c r="I28">
-        <f>SUBTOTAL(9,I3:I27)</f>
+        <f t="shared" si="0"/>
         <v>8730</v>
       </c>
       <c r="J28">
-        <f>SUBTOTAL(9,J3:J27)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="K28">
-        <f>SUBTOTAL(9,K3:K27)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L28">
-        <f>SUBTOTAL(9,L3:L27)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="M28">
-        <f>SUBTOTAL(9,M3:M27)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="N28">
-        <f>SUBTOTAL(9,N3:N27)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="O28">
-        <f>SUBTOTAL(9,O3:O27)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="P28">
-        <f>SUBTOTAL(9,P3:P27)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q28">
-        <f>SUBTOTAL(9,Q3:Q27)</f>
+        <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="R28">
-        <f>SUBTOTAL(9,R3:R27)</f>
-        <v>120</v>
+        <f t="shared" si="0"/>
+        <v>150</v>
       </c>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.25">
       <c r="I29" s="29">
         <v>-1450</v>
       </c>
-      <c r="J29" s="30" t="s">
+      <c r="J29" s="22" t="s">
         <v>329</v>
       </c>
     </row>
@@ -26307,7 +26308,7 @@
       </c>
       <c r="I34" s="13">
         <f>R28</f>
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="J34" s="14"/>
     </row>
@@ -26361,7 +26362,7 @@
       </c>
       <c r="I40" s="19">
         <f>SUM(I33:I39)</f>
-        <v>7400</v>
+        <v>7430</v>
       </c>
       <c r="J40" s="19">
         <f>SUM(J33:J37)</f>
@@ -26414,34 +26415,34 @@
       </c>
     </row>
     <row r="44" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="31" t="s">
+      <c r="A44" s="30" t="s">
         <v>2051</v>
       </c>
-      <c r="B44" s="31" t="s">
+      <c r="B44" s="30" t="s">
         <v>2052</v>
       </c>
-      <c r="C44" s="31" t="s">
+      <c r="C44" s="30" t="s">
         <v>2053</v>
       </c>
-      <c r="D44" s="32">
+      <c r="D44" s="31">
         <v>7</v>
       </c>
-      <c r="E44" s="33">
+      <c r="E44" s="32">
         <v>1320</v>
       </c>
-      <c r="F44" s="33">
+      <c r="F44" s="32">
         <v>0</v>
       </c>
-      <c r="G44" s="33">
+      <c r="G44" s="32">
         <v>1320</v>
       </c>
-      <c r="H44" s="31" t="s">
+      <c r="H44" s="30" t="s">
         <v>2054</v>
       </c>
-      <c r="I44" s="31" t="s">
-        <v>25</v>
-      </c>
-      <c r="J44" s="31" t="s">
+      <c r="I44" s="30" t="s">
+        <v>25</v>
+      </c>
+      <c r="J44" s="30" t="s">
         <v>2048</v>
       </c>
       <c r="K44" s="3" t="s">

</xml_diff>

<commit_message>
Final report for March
</commit_message>
<xml_diff>
--- a/data/Mar/THÁNG 3.2026- CHÂU NGÂN- ĐỐI SOÁT.xlsx
+++ b/data/Mar/THÁNG 3.2026- CHÂU NGÂN- ĐỐI SOÁT.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Freelance\TextInputter\data\Mar\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\TextExtractorTool\data\Mar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F949A4F5-1D2B-4D0B-BA1A-F802C936D4F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{201D6C93-A636-49C1-8662-9B053CA08085}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="8" activeTab="24" xr2:uid="{5C19E60F-B0EA-4466-8994-298A0AC29210}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{5C19E60F-B0EA-4466-8994-298A0AC29210}"/>
   </bookViews>
   <sheets>
     <sheet name="2-3" sheetId="1" r:id="rId1"/>
@@ -9145,7 +9145,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -9222,6 +9222,7 @@
     <xf numFmtId="0" fontId="8" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -24970,7 +24971,7 @@
       <c r="N3" s="5"/>
       <c r="O3" s="5"/>
       <c r="P3" s="5"/>
-      <c r="Q3" s="4">
+      <c r="Q3" s="50">
         <v>1</v>
       </c>
     </row>
@@ -25015,7 +25016,7 @@
       <c r="N4" s="5"/>
       <c r="O4" s="5"/>
       <c r="P4" s="5"/>
-      <c r="Q4">
+      <c r="Q4" s="50">
         <v>1</v>
       </c>
     </row>
@@ -25058,7 +25059,7 @@
       <c r="N5" s="5"/>
       <c r="O5" s="5"/>
       <c r="P5" s="5"/>
-      <c r="Q5">
+      <c r="Q5" s="50">
         <v>1</v>
       </c>
     </row>
@@ -25101,7 +25102,7 @@
       <c r="N6" s="5"/>
       <c r="O6" s="5"/>
       <c r="P6" s="5"/>
-      <c r="Q6">
+      <c r="Q6" s="50">
         <v>1</v>
       </c>
     </row>
@@ -25144,7 +25145,7 @@
       <c r="N7" s="21"/>
       <c r="O7" s="21"/>
       <c r="P7" s="21"/>
-      <c r="Q7" s="22">
+      <c r="Q7" s="42">
         <v>1</v>
       </c>
       <c r="R7" s="22">
@@ -25193,7 +25194,7 @@
       <c r="N8" s="5"/>
       <c r="O8" s="5"/>
       <c r="P8" s="5"/>
-      <c r="Q8">
+      <c r="Q8" s="50">
         <v>1</v>
       </c>
       <c r="R8" s="22">
@@ -25240,7 +25241,7 @@
       <c r="N9" s="5"/>
       <c r="O9" s="5"/>
       <c r="P9" s="5"/>
-      <c r="Q9">
+      <c r="Q9" s="50">
         <v>1</v>
       </c>
     </row>
@@ -25285,7 +25286,7 @@
       <c r="N10" s="5"/>
       <c r="O10" s="5"/>
       <c r="P10" s="5"/>
-      <c r="Q10">
+      <c r="Q10" s="50">
         <v>1</v>
       </c>
     </row>
@@ -25328,7 +25329,7 @@
       <c r="N11" s="5"/>
       <c r="O11" s="5"/>
       <c r="P11" s="5"/>
-      <c r="Q11">
+      <c r="Q11" s="50">
         <v>1</v>
       </c>
     </row>
@@ -25371,7 +25372,7 @@
       <c r="N12" s="5"/>
       <c r="O12" s="5"/>
       <c r="P12" s="5"/>
-      <c r="Q12">
+      <c r="Q12" s="50">
         <v>1</v>
       </c>
     </row>
@@ -25414,7 +25415,7 @@
       <c r="N13" s="5"/>
       <c r="O13" s="5"/>
       <c r="P13" s="5"/>
-      <c r="Q13">
+      <c r="Q13" s="50">
         <v>1</v>
       </c>
       <c r="R13" s="22">
@@ -25461,7 +25462,7 @@
       <c r="N14" s="5"/>
       <c r="O14" s="5"/>
       <c r="P14" s="5"/>
-      <c r="Q14">
+      <c r="Q14" s="50">
         <v>1</v>
       </c>
     </row>
@@ -25504,7 +25505,7 @@
       <c r="N15" s="5"/>
       <c r="O15" s="5"/>
       <c r="P15" s="5"/>
-      <c r="Q15">
+      <c r="Q15" s="50">
         <v>1</v>
       </c>
     </row>
@@ -25547,7 +25548,7 @@
       <c r="N16" s="5"/>
       <c r="O16" s="5"/>
       <c r="P16" s="5"/>
-      <c r="Q16">
+      <c r="Q16" s="50">
         <v>1</v>
       </c>
     </row>
@@ -25590,7 +25591,7 @@
       <c r="N17" s="5"/>
       <c r="O17" s="5"/>
       <c r="P17" s="5"/>
-      <c r="Q17">
+      <c r="Q17" s="50">
         <v>1</v>
       </c>
       <c r="R17" s="22">
@@ -25637,7 +25638,7 @@
       <c r="N18" s="5"/>
       <c r="O18" s="5"/>
       <c r="P18" s="5"/>
-      <c r="Q18">
+      <c r="Q18" s="50">
         <v>1</v>
       </c>
     </row>
@@ -25680,7 +25681,7 @@
       <c r="N19" s="5"/>
       <c r="O19" s="5"/>
       <c r="P19" s="5"/>
-      <c r="Q19">
+      <c r="Q19" s="50">
         <v>1</v>
       </c>
     </row>
@@ -25723,7 +25724,7 @@
       <c r="N20" s="5"/>
       <c r="O20" s="5"/>
       <c r="P20" s="5"/>
-      <c r="Q20">
+      <c r="Q20" s="50">
         <v>1</v>
       </c>
     </row>
@@ -25766,7 +25767,7 @@
       <c r="N21" s="5"/>
       <c r="O21" s="5"/>
       <c r="P21" s="5"/>
-      <c r="Q21">
+      <c r="Q21" s="50">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update report 10-04 and constants
</commit_message>
<xml_diff>
--- a/data/Mar/THÁNG 3.2026- CHÂU NGÂN- ĐỐI SOÁT.xlsx
+++ b/data/Mar/THÁNG 3.2026- CHÂU NGÂN- ĐỐI SOÁT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Freelance\TextInputter\data\Mar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22F46BE4-0E34-4645-A82F-83EEC2D62E87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{967116A2-038C-4333-A5E6-7CBD1C67E161}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="9" activeTab="25" xr2:uid="{5C19E60F-B0EA-4466-8994-298A0AC29210}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="6" activeTab="6" xr2:uid="{5C19E60F-B0EA-4466-8994-298A0AC29210}"/>
   </bookViews>
   <sheets>
     <sheet name="2-3" sheetId="1" r:id="rId1"/>
@@ -26202,6 +26202,7 @@
     <col min="1" max="2" width="9.140625" customWidth="1"/>
     <col min="3" max="3" width="30" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">

</xml_diff>